<commit_message>
. Updated the gamedatabase
</commit_message>
<xml_diff>
--- a/games_database.xlsx
+++ b/games_database.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\azree\OneDrive\Desktop\Github Repro\Capstone\JustAnotherDiscordRichPresenceApp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBFA44C3-8297-42B1-B260-96E45C5AD714}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91447F69-79AE-4254-A753-321118D09B8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5282" uniqueCount="1917">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5289" uniqueCount="1924">
   <si>
     <t>Game Title</t>
   </si>
@@ -5783,6 +5783,27 @@
   </si>
   <si>
     <t>Assault: Retribution</t>
+  </si>
+  <si>
+    <t>King's Field</t>
+  </si>
+  <si>
+    <t>King's Field II</t>
+  </si>
+  <si>
+    <t>King's Field III</t>
+  </si>
+  <si>
+    <t>Shadow Tower</t>
+  </si>
+  <si>
+    <t>Echo Night</t>
+  </si>
+  <si>
+    <t>Echo Night 2: The Lord of Nightmares</t>
+  </si>
+  <si>
+    <t>Spriggan: Lunar Verse</t>
   </si>
 </sst>
 </file>
@@ -6291,7 +6312,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FFEDB219-5142-4DD7-A4D0-88AB6C946699}">
-  <dimension ref="A1:G58"/>
+  <dimension ref="A1:G65"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="24.88671875" bestFit="1" customWidth="1"/>
@@ -6852,6 +6873,41 @@
     <row r="58" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>1916</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A59" t="s">
+        <v>1917</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A60" t="s">
+        <v>1918</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A61" t="s">
+        <v>1919</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A62" t="s">
+        <v>1920</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A63" t="s">
+        <v>1921</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A64" t="s">
+        <v>1922</v>
+      </c>
+    </row>
+    <row r="65" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A65" t="s">
+        <v>1923</v>
       </c>
     </row>
   </sheetData>

</xml_diff>